<commit_message>
Defect balance seems working for both discrete and bin-moments
</commit_message>
<xml_diff>
--- a/Expanded_Eurofer_CD/input/input_parameters.xlsx
+++ b/Expanded_Eurofer_CD/input/input_parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Owner\Documents\Repos\EuroferMicrostructure\Expanded_Eurofer_CD\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D56175FA-2106-4A85-90F3-42DC12A6D58F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90F6D56D-5E48-4DE1-AFFF-2E51F856C8DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="591" uniqueCount="406">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="408">
   <si>
     <t>Parameter</t>
   </si>
@@ -1242,6 +1242,12 @@
   </si>
   <si>
     <t>gmres</t>
+  </si>
+  <si>
+    <t>shape_function</t>
+  </si>
+  <si>
+    <t>lognormal</t>
   </si>
 </sst>
 </file>
@@ -1702,10 +1708,10 @@
         <v>20</v>
       </c>
       <c r="C7">
-        <v>0.57999999999999996</v>
+        <v>0.25</v>
       </c>
       <c r="D7">
-        <v>0.65</v>
+        <v>0.35</v>
       </c>
       <c r="E7" t="s">
         <v>8</v>
@@ -1775,10 +1781,10 @@
         <v>30</v>
       </c>
       <c r="C12">
-        <v>0.15</v>
+        <v>0.05</v>
       </c>
       <c r="D12">
-        <v>0.2</v>
+        <v>0.08</v>
       </c>
       <c r="E12" t="s">
         <v>8</v>
@@ -2441,7 +2447,7 @@
         <v>129</v>
       </c>
       <c r="C11">
-        <v>0.03</v>
+        <v>0.34</v>
       </c>
       <c r="D11" t="s">
         <v>65</v>
@@ -3111,7 +3117,7 @@
         <v>224</v>
       </c>
       <c r="C19">
-        <v>0.75009999999999999</v>
+        <v>3</v>
       </c>
       <c r="D19" t="s">
         <v>65</v>
@@ -3139,7 +3145,7 @@
         <v>228</v>
       </c>
       <c r="C21">
-        <v>0.71599999999999997</v>
+        <v>3</v>
       </c>
       <c r="D21" t="s">
         <v>65</v>
@@ -3466,7 +3472,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="31.1796875" style="3" customWidth="1"/>
@@ -3594,7 +3600,7 @@
         <v>292</v>
       </c>
       <c r="C9" s="5">
-        <v>1000000000000</v>
+        <v>10000000000000</v>
       </c>
       <c r="D9" t="s">
         <v>293</v>
@@ -3688,8 +3694,8 @@
       <c r="B16" t="s">
         <v>309</v>
       </c>
-      <c r="C16">
-        <v>0</v>
+      <c r="C16" s="5">
+        <v>1E+20</v>
       </c>
       <c r="D16" t="s">
         <v>310</v>
@@ -3705,8 +3711,8 @@
       <c r="B17" t="s">
         <v>313</v>
       </c>
-      <c r="C17">
-        <v>5.0000000000000001E-9</v>
+      <c r="C17" s="5">
+        <v>4.9999999999999998E-8</v>
       </c>
       <c r="D17" t="s">
         <v>305</v>
@@ -3803,7 +3809,7 @@
         <v>327</v>
       </c>
       <c r="C25">
-        <v>500</v>
+        <v>10000</v>
       </c>
       <c r="D25" t="s">
         <v>8</v>
@@ -3820,7 +3826,7 @@
         <v>330</v>
       </c>
       <c r="C26">
-        <v>500</v>
+        <v>10000</v>
       </c>
       <c r="D26" t="s">
         <v>8</v>
@@ -4025,7 +4031,7 @@
         <v>367</v>
       </c>
       <c r="C40" s="5">
-        <v>1E-4</v>
+        <v>9.9999999999999995E-7</v>
       </c>
       <c r="D40" t="s">
         <v>8</v>
@@ -4039,7 +4045,7 @@
         <v>369</v>
       </c>
       <c r="C41" s="5">
-        <v>9.9999999999999995E-21</v>
+        <v>1E-25</v>
       </c>
       <c r="D41" t="s">
         <v>8</v>
@@ -4191,7 +4197,7 @@
         <v>394</v>
       </c>
       <c r="C51">
-        <v>600</v>
+        <v>573</v>
       </c>
       <c r="D51" t="s">
         <v>395</v>
@@ -4207,7 +4213,7 @@
       <c r="B52" t="s">
         <v>397</v>
       </c>
-      <c r="C52">
+      <c r="C52" s="5">
         <v>9.9999999999999995E-7</v>
       </c>
       <c r="D52" t="s">
@@ -4246,6 +4252,14 @@
       </c>
       <c r="E54" t="s">
         <v>404</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B55" t="s">
+        <v>406</v>
+      </c>
+      <c r="C55" t="s">
+        <v>407</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
completed sliding window and openMP
</commit_message>
<xml_diff>
--- a/Expanded_Eurofer_CD/input/input_parameters.xlsx
+++ b/Expanded_Eurofer_CD/input/input_parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Owner\Documents\Repos\EuroferMicrostructure\Expanded_Eurofer_CD\input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ghoni/Documents/GitHub/EuroferMicrostructure/Expanded_Eurofer_CD/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90F6D56D-5E48-4DE1-AFFF-2E51F856C8DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CB8DAB6-17CB-4748-AF60-2381862DD239}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20260" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Production" sheetId="1" r:id="rId1"/>
@@ -1263,18 +1263,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -1312,8 +1306,8 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1617,12 +1611,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="32.453125" customWidth="1"/>
+    <col min="1" max="1" width="32.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1639,12 +1633,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -1661,7 +1655,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1678,7 +1672,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -1695,12 +1689,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -1717,7 +1711,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -1734,7 +1728,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>23</v>
       </c>
@@ -1751,7 +1745,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>26</v>
       </c>
@@ -1768,12 +1762,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>29</v>
       </c>
@@ -1790,7 +1784,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -1807,7 +1801,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>33</v>
       </c>
@@ -1824,7 +1818,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>36</v>
       </c>
@@ -1849,12 +1843,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E31"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="28.36328125" customWidth="1"/>
+    <col min="1" max="1" width="28.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1871,12 +1865,12 @@
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>41</v>
       </c>
@@ -1893,7 +1887,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>45</v>
       </c>
@@ -1910,7 +1904,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>49</v>
       </c>
@@ -1924,7 +1918,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>51</v>
       </c>
@@ -1938,7 +1932,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>53</v>
       </c>
@@ -1952,7 +1946,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>56</v>
       </c>
@@ -1966,7 +1960,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>58</v>
       </c>
@@ -1983,12 +1977,12 @@
         <v>61</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>63</v>
       </c>
@@ -2005,7 +1999,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>67</v>
       </c>
@@ -2022,7 +2016,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>70</v>
       </c>
@@ -2039,7 +2033,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>73</v>
       </c>
@@ -2056,12 +2050,12 @@
         <v>72</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>76</v>
       </c>
@@ -2078,7 +2072,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>78</v>
       </c>
@@ -2095,7 +2089,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>81</v>
       </c>
@@ -2112,7 +2106,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>83</v>
       </c>
@@ -2129,12 +2123,12 @@
         <v>72</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>86</v>
       </c>
@@ -2151,7 +2145,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>88</v>
       </c>
@@ -2168,7 +2162,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>91</v>
       </c>
@@ -2185,7 +2179,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>93</v>
       </c>
@@ -2202,12 +2196,12 @@
         <v>90</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>96</v>
       </c>
@@ -2221,7 +2215,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>99</v>
       </c>
@@ -2235,7 +2229,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>101</v>
       </c>
@@ -2249,12 +2243,12 @@
         <v>98</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>104</v>
       </c>
@@ -2271,7 +2265,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>108</v>
       </c>
@@ -2296,13 +2290,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E40"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="37.6328125" customWidth="1"/>
-    <col min="2" max="2" width="18.08984375" customWidth="1"/>
+    <col min="1" max="1" width="37.6640625" customWidth="1"/>
+    <col min="2" max="2" width="18.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2319,12 +2313,12 @@
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>113</v>
       </c>
@@ -2341,7 +2335,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>117</v>
       </c>
@@ -2355,7 +2349,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>118</v>
       </c>
@@ -2372,7 +2366,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>120</v>
       </c>
@@ -2386,7 +2380,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>121</v>
       </c>
@@ -2403,7 +2397,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>123</v>
       </c>
@@ -2417,12 +2411,12 @@
         <v>65</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>125</v>
       </c>
@@ -2439,7 +2433,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>128</v>
       </c>
@@ -2456,7 +2450,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>131</v>
       </c>
@@ -2473,7 +2467,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>134</v>
       </c>
@@ -2487,12 +2481,12 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>131</v>
       </c>
@@ -2506,7 +2500,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>134</v>
       </c>
@@ -2520,12 +2514,12 @@
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>140</v>
       </c>
@@ -2542,7 +2536,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>144</v>
       </c>
@@ -2559,7 +2553,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>147</v>
       </c>
@@ -2576,7 +2570,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>150</v>
       </c>
@@ -2593,7 +2587,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>153</v>
       </c>
@@ -2610,12 +2604,12 @@
         <v>152</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>156</v>
       </c>
@@ -2632,7 +2626,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>159</v>
       </c>
@@ -2649,7 +2643,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>161</v>
       </c>
@@ -2666,7 +2660,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>164</v>
       </c>
@@ -2683,12 +2677,12 @@
         <v>166</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>168</v>
       </c>
@@ -2705,7 +2699,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>171</v>
       </c>
@@ -2722,7 +2716,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>173</v>
       </c>
@@ -2739,7 +2733,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>175</v>
       </c>
@@ -2756,7 +2750,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>177</v>
       </c>
@@ -2773,12 +2767,12 @@
         <v>163</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>180</v>
       </c>
@@ -2795,7 +2789,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>183</v>
       </c>
@@ -2812,7 +2806,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>185</v>
       </c>
@@ -2829,12 +2823,12 @@
         <v>158</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>188</v>
       </c>
@@ -2851,7 +2845,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>191</v>
       </c>
@@ -2876,35 +2870,35 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E43"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="40" style="1" customWidth="1"/>
+    <col min="1" max="1" width="40" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" s="5" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" s="5" t="s">
         <v>195</v>
       </c>
       <c r="B3" t="s">
@@ -2917,8 +2911,8 @@
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" s="5" t="s">
         <v>58</v>
       </c>
       <c r="B4" t="s">
@@ -2931,8 +2925,8 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" s="5" t="s">
         <v>196</v>
       </c>
       <c r="B5" t="s">
@@ -2948,8 +2942,8 @@
         <v>198</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" s="5" t="s">
         <v>199</v>
       </c>
       <c r="B6" t="s">
@@ -2965,13 +2959,13 @@
         <v>202</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" s="5" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A8" s="1" t="s">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" s="5" t="s">
         <v>204</v>
       </c>
       <c r="B8" t="s">
@@ -2987,8 +2981,8 @@
         <v>206</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A9" s="1" t="s">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" s="5" t="s">
         <v>207</v>
       </c>
       <c r="B9" t="s">
@@ -3001,8 +2995,8 @@
         <v>65</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A10" s="1" t="s">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" s="5" t="s">
         <v>209</v>
       </c>
       <c r="B10" t="s">
@@ -3015,8 +3009,8 @@
         <v>65</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A11" s="1" t="s">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" s="5" t="s">
         <v>211</v>
       </c>
       <c r="B11" t="s">
@@ -3029,8 +3023,8 @@
         <v>65</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A12" s="1" t="s">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" s="5" t="s">
         <v>213</v>
       </c>
       <c r="B12" t="s">
@@ -3043,13 +3037,13 @@
         <v>65</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A13" s="1" t="s">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" s="5" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A14" s="1" t="s">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" s="5" t="s">
         <v>216</v>
       </c>
       <c r="B14" t="s">
@@ -3062,8 +3056,8 @@
         <v>60</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A15" s="1" t="s">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" s="5" t="s">
         <v>218</v>
       </c>
       <c r="B15" t="s">
@@ -3076,8 +3070,8 @@
         <v>50</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A16" s="1" t="s">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" s="5" t="s">
         <v>220</v>
       </c>
       <c r="B16" t="s">
@@ -3090,8 +3084,8 @@
         <v>65</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A17" s="1" t="s">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" s="5" t="s">
         <v>199</v>
       </c>
       <c r="B17" t="s">
@@ -3104,13 +3098,13 @@
         <v>201</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A18" s="1" t="s">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" s="5" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A19" s="1" t="s">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" s="5" t="s">
         <v>223</v>
       </c>
       <c r="B19" t="s">
@@ -3123,8 +3117,8 @@
         <v>65</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A20" s="1" t="s">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" s="5" t="s">
         <v>225</v>
       </c>
       <c r="B20" t="s">
@@ -3137,8 +3131,8 @@
         <v>8</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A21" s="1" t="s">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21" s="5" t="s">
         <v>227</v>
       </c>
       <c r="B21" t="s">
@@ -3151,8 +3145,8 @@
         <v>65</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A22" s="1" t="s">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A22" s="5" t="s">
         <v>229</v>
       </c>
       <c r="B22" t="s">
@@ -3165,8 +3159,8 @@
         <v>8</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A23" s="1" t="s">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A23" s="5" t="s">
         <v>231</v>
       </c>
       <c r="B23" t="s">
@@ -3179,8 +3173,8 @@
         <v>25</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A24" s="1" t="s">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24" s="5" t="s">
         <v>233</v>
       </c>
       <c r="B24" t="s">
@@ -3193,13 +3187,13 @@
         <v>25</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A25" s="1" t="s">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A25" s="5" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A26" s="1" t="s">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A26" s="5" t="s">
         <v>236</v>
       </c>
       <c r="B26" t="s">
@@ -3215,13 +3209,13 @@
         <v>238</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A27" s="1" t="s">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A27" s="5" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A28" s="1" t="s">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A28" s="5" t="s">
         <v>240</v>
       </c>
       <c r="B28" t="s">
@@ -3237,8 +3231,8 @@
         <v>243</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A29" s="1" t="s">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A29" s="5" t="s">
         <v>244</v>
       </c>
       <c r="B29" t="s">
@@ -3254,8 +3248,8 @@
         <v>245</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A30" s="1" t="s">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A30" s="5" t="s">
         <v>246</v>
       </c>
       <c r="B30" t="s">
@@ -3271,13 +3265,13 @@
         <v>245</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A31" s="1" t="s">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A31" s="5" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A32" s="1" t="s">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A32" s="5" t="s">
         <v>199</v>
       </c>
       <c r="B32" t="s">
@@ -3293,8 +3287,8 @@
         <v>250</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A33" s="1" t="s">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A33" s="5" t="s">
         <v>251</v>
       </c>
       <c r="B33" t="s">
@@ -3310,8 +3304,8 @@
         <v>253</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A34" s="1" t="s">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A34" s="5" t="s">
         <v>254</v>
       </c>
       <c r="B34" t="s">
@@ -3327,8 +3321,8 @@
         <v>253</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A35" s="1" t="s">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A35" s="5" t="s">
         <v>256</v>
       </c>
       <c r="B35" t="s">
@@ -3344,13 +3338,13 @@
         <v>253</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A36" s="1" t="s">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A36" s="5" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A37" s="1" t="s">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A37" s="5" t="s">
         <v>125</v>
       </c>
       <c r="B37" t="s">
@@ -3363,8 +3357,8 @@
         <v>98</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A38" s="1" t="s">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A38" s="5" t="s">
         <v>260</v>
       </c>
       <c r="B38" t="s">
@@ -3380,8 +3374,8 @@
         <v>262</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A39" s="1" t="s">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A39" s="5" t="s">
         <v>263</v>
       </c>
       <c r="B39" t="s">
@@ -3397,8 +3391,8 @@
         <v>262</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A40" s="1" t="s">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A40" s="5" t="s">
         <v>265</v>
       </c>
       <c r="B40" t="s">
@@ -3414,8 +3408,8 @@
         <v>267</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A41" s="1" t="s">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A41" s="5" t="s">
         <v>268</v>
       </c>
       <c r="B41" t="s">
@@ -3431,8 +3425,8 @@
         <v>270</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A42" s="1" t="s">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A42" s="5" t="s">
         <v>271</v>
       </c>
       <c r="B42" t="s">
@@ -3448,8 +3442,8 @@
         <v>270</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A43" s="1" t="s">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A43" s="5" t="s">
         <v>273</v>
       </c>
       <c r="B43" t="s">
@@ -3473,37 +3467,37 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:E55"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="31.1796875" style="3" customWidth="1"/>
-    <col min="2" max="2" width="13.36328125" customWidth="1"/>
-    <col min="3" max="3" width="16.453125" customWidth="1"/>
+    <col min="1" max="1" width="31.1640625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="13.33203125" customWidth="1"/>
+    <col min="3" max="3" width="16.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
         <v>276</v>
       </c>
       <c r="B3" t="s">
@@ -3519,8 +3513,8 @@
         <v>278</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
         <v>279</v>
       </c>
       <c r="B4" t="s">
@@ -3536,8 +3530,8 @@
         <v>281</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
         <v>282</v>
       </c>
       <c r="B5" t="s">
@@ -3553,8 +3547,8 @@
         <v>284</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
         <v>285</v>
       </c>
       <c r="B6" t="s">
@@ -3570,8 +3564,8 @@
         <v>286</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
         <v>287</v>
       </c>
       <c r="B7" t="s">
@@ -3587,19 +3581,19 @@
         <v>289</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A8" s="3" t="s">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A9" s="3" t="s">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
         <v>291</v>
       </c>
       <c r="B9" t="s">
         <v>292</v>
       </c>
-      <c r="C9" s="5">
+      <c r="C9" s="4">
         <v>10000000000000</v>
       </c>
       <c r="D9" t="s">
@@ -3609,8 +3603,8 @@
         <v>294</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A10" s="3" t="s">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
         <v>295</v>
       </c>
       <c r="B10" t="s">
@@ -3626,8 +3620,8 @@
         <v>297</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A11" s="3" t="s">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
         <v>298</v>
       </c>
       <c r="B11" t="s">
@@ -3643,8 +3637,8 @@
         <v>297</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A12" s="3" t="s">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
         <v>300</v>
       </c>
       <c r="B12" t="s">
@@ -3660,19 +3654,19 @@
         <v>297</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A13" s="3" t="s">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A14" s="3" t="s">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
         <v>303</v>
       </c>
       <c r="B14" t="s">
         <v>304</v>
       </c>
-      <c r="C14" s="5">
+      <c r="C14" s="4">
         <v>1E-3</v>
       </c>
       <c r="D14" t="s">
@@ -3682,19 +3676,19 @@
         <v>306</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A15" s="3" t="s">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A16" s="3" t="s">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" s="2" t="s">
         <v>308</v>
       </c>
       <c r="B16" t="s">
         <v>309</v>
       </c>
-      <c r="C16" s="5">
+      <c r="C16" s="4">
         <v>1E+20</v>
       </c>
       <c r="D16" t="s">
@@ -3704,14 +3698,14 @@
         <v>311</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A17" s="3" t="s">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" s="2" t="s">
         <v>312</v>
       </c>
       <c r="B17" t="s">
         <v>313</v>
       </c>
-      <c r="C17" s="5">
+      <c r="C17" s="4">
         <v>4.9999999999999998E-8</v>
       </c>
       <c r="D17" t="s">
@@ -3721,8 +3715,8 @@
         <v>306</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A18" s="3" t="s">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" s="2" t="s">
         <v>314</v>
       </c>
       <c r="B18" t="s">
@@ -3735,8 +3729,8 @@
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A19" s="3" t="s">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" s="2" t="s">
         <v>316</v>
       </c>
       <c r="B19" t="s">
@@ -3749,13 +3743,13 @@
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A20" s="3" t="s">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" s="2" t="s">
         <v>318</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A21" s="3" t="s">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21" s="2" t="s">
         <v>319</v>
       </c>
       <c r="B21" t="s">
@@ -3768,8 +3762,8 @@
         <v>321</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A22" s="3" t="s">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A22" s="2" t="s">
         <v>322</v>
       </c>
       <c r="B22" t="s">
@@ -3782,13 +3776,13 @@
         <v>321</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A23" s="3" t="s">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A23" s="2" t="s">
         <v>324</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A24" s="3" t="s">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24" s="2" t="s">
         <v>325</v>
       </c>
       <c r="B24" t="s">
@@ -3801,8 +3795,8 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A25" s="3" t="s">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A25" s="2" t="s">
         <v>326</v>
       </c>
       <c r="B25" t="s">
@@ -3818,8 +3812,8 @@
         <v>328</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A26" s="3" t="s">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A26" s="2" t="s">
         <v>329</v>
       </c>
       <c r="B26" t="s">
@@ -3835,8 +3829,8 @@
         <v>328</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A27" s="3" t="s">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A27" s="2" t="s">
         <v>331</v>
       </c>
       <c r="B27" t="s">
@@ -3852,13 +3846,13 @@
         <v>334</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A28" s="3" t="s">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A28" s="2" t="s">
         <v>335</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A29" s="3" t="s">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A29" s="2" t="s">
         <v>336</v>
       </c>
       <c r="B29" t="s">
@@ -3874,8 +3868,8 @@
         <v>338</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A30" s="3" t="s">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A30" s="2" t="s">
         <v>339</v>
       </c>
       <c r="B30" t="s">
@@ -3891,8 +3885,8 @@
         <v>341</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A31" s="3" t="s">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A31" s="2" t="s">
         <v>342</v>
       </c>
       <c r="B31" t="s">
@@ -3908,8 +3902,8 @@
         <v>338</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A32" s="3" t="s">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A32" s="2" t="s">
         <v>344</v>
       </c>
       <c r="B32" t="s">
@@ -3925,13 +3919,13 @@
         <v>346</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A33" s="3" t="s">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A33" s="2" t="s">
         <v>347</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A34" s="3" t="s">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A34" s="2" t="s">
         <v>348</v>
       </c>
       <c r="B34" t="s">
@@ -3947,8 +3941,8 @@
         <v>351</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A35" s="3" t="s">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A35" s="2" t="s">
         <v>352</v>
       </c>
       <c r="B35" t="s">
@@ -3964,8 +3958,8 @@
         <v>355</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A36" s="3" t="s">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A36" s="2" t="s">
         <v>356</v>
       </c>
       <c r="B36" t="s">
@@ -3978,8 +3972,8 @@
         <v>358</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A37" s="3" t="s">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A37" s="2" t="s">
         <v>359</v>
       </c>
       <c r="B37" t="s">
@@ -3992,8 +3986,8 @@
         <v>358</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A38" s="3" t="s">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A38" s="2" t="s">
         <v>361</v>
       </c>
       <c r="B38" t="s">
@@ -4006,8 +4000,8 @@
         <v>8</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A39" s="3" t="s">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A39" s="2" t="s">
         <v>363</v>
       </c>
       <c r="B39" t="s">
@@ -4023,36 +4017,36 @@
         <v>365</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A40" s="3" t="s">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A40" s="2" t="s">
         <v>366</v>
       </c>
       <c r="B40" t="s">
         <v>367</v>
       </c>
-      <c r="C40" s="5">
+      <c r="C40" s="4">
         <v>9.9999999999999995E-7</v>
       </c>
       <c r="D40" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A41" s="3" t="s">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A41" s="2" t="s">
         <v>368</v>
       </c>
       <c r="B41" t="s">
         <v>369</v>
       </c>
-      <c r="C41" s="5">
+      <c r="C41" s="4">
         <v>1E-25</v>
       </c>
       <c r="D41" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A42" s="3" t="s">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A42" s="2" t="s">
         <v>370</v>
       </c>
       <c r="B42" t="s">
@@ -4068,8 +4062,8 @@
         <v>372</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A43" s="3" t="s">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A43" s="2" t="s">
         <v>373</v>
       </c>
       <c r="B43" t="s">
@@ -4085,8 +4079,8 @@
         <v>375</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A44" s="3" t="s">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A44" s="2" t="s">
         <v>376</v>
       </c>
       <c r="B44" t="s">
@@ -4102,8 +4096,8 @@
         <v>375</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A45" s="3" t="s">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A45" s="2" t="s">
         <v>378</v>
       </c>
       <c r="B45" t="s">
@@ -4119,8 +4113,8 @@
         <v>380</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A46" s="3" t="s">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A46" s="2" t="s">
         <v>381</v>
       </c>
       <c r="B46" t="s">
@@ -4136,8 +4130,8 @@
         <v>383</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A47" s="3" t="s">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A47" s="2" t="s">
         <v>384</v>
       </c>
       <c r="B47" t="s">
@@ -4153,8 +4147,8 @@
         <v>386</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A48" s="3" t="s">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A48" s="2" t="s">
         <v>387</v>
       </c>
       <c r="B48" t="s">
@@ -4170,8 +4164,8 @@
         <v>389</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A49" s="3" t="s">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A49" s="2" t="s">
         <v>390</v>
       </c>
       <c r="B49" t="s">
@@ -4184,13 +4178,13 @@
         <v>8</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A50" s="3" t="s">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A50" s="2" t="s">
         <v>392</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A51" s="3" t="s">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A51" s="2" t="s">
         <v>393</v>
       </c>
       <c r="B51" t="s">
@@ -4206,22 +4200,22 @@
         <v>396</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A52" s="3" t="s">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A52" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B52" t="s">
         <v>397</v>
       </c>
-      <c r="C52" s="5">
+      <c r="C52" s="4">
         <v>9.9999999999999995E-7</v>
       </c>
       <c r="D52" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A53" s="3" t="s">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A53" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B53" t="s">
@@ -4237,8 +4231,8 @@
         <v>400</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A54" s="3" t="s">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A54" s="2" t="s">
         <v>401</v>
       </c>
       <c r="B54" t="s">
@@ -4254,7 +4248,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B55" t="s">
         <v>406</v>
       </c>

</xml_diff>

<commit_message>
Added Woodbury preconditioner for large systems. Fixed all defect imbalances
</commit_message>
<xml_diff>
--- a/Expanded_Eurofer_CD/input/input_parameters.xlsx
+++ b/Expanded_Eurofer_CD/input/input_parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ghoni/Documents/GitHub/EuroferMicrostructure/Expanded_Eurofer_CD/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CB8DAB6-17CB-4748-AF60-2381862DD239}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{526E54FF-4042-144B-88DB-DC7701DBB4C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20260" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4440" yWindow="760" windowWidth="24960" windowHeight="16820" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Production" sheetId="1" r:id="rId1"/>
@@ -1301,13 +1301,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2458,7 +2457,7 @@
         <v>132</v>
       </c>
       <c r="C12">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="D12" t="s">
         <v>8</v>
@@ -2617,7 +2616,7 @@
         <v>157</v>
       </c>
       <c r="C24">
-        <v>0.45</v>
+        <v>0.6</v>
       </c>
       <c r="D24" t="s">
         <v>65</v>
@@ -2634,7 +2633,7 @@
         <v>160</v>
       </c>
       <c r="C25">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="D25" t="s">
         <v>65</v>
@@ -2780,7 +2779,7 @@
         <v>181</v>
       </c>
       <c r="C35">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="D35" t="s">
         <v>65</v>
@@ -2797,7 +2796,7 @@
         <v>184</v>
       </c>
       <c r="C36">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="D36" t="s">
         <v>65</v>
@@ -2872,11 +2871,11 @@
   <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="40" style="5" customWidth="1"/>
+    <col min="1" max="1" width="40" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="5" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -2893,12 +2892,12 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" s="5" t="s">
+      <c r="A2" t="s">
         <v>194</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" s="5" t="s">
+      <c r="A3" t="s">
         <v>195</v>
       </c>
       <c r="B3" t="s">
@@ -2912,7 +2911,7 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" s="5" t="s">
+      <c r="A4" t="s">
         <v>58</v>
       </c>
       <c r="B4" t="s">
@@ -2926,7 +2925,7 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="5" t="s">
+      <c r="A5" t="s">
         <v>196</v>
       </c>
       <c r="B5" t="s">
@@ -2943,7 +2942,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="5" t="s">
+      <c r="A6" t="s">
         <v>199</v>
       </c>
       <c r="B6" t="s">
@@ -2960,12 +2959,12 @@
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="5" t="s">
+      <c r="A7" t="s">
         <v>203</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" s="5" t="s">
+      <c r="A8" t="s">
         <v>204</v>
       </c>
       <c r="B8" t="s">
@@ -2982,7 +2981,7 @@
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" s="5" t="s">
+      <c r="A9" t="s">
         <v>207</v>
       </c>
       <c r="B9" t="s">
@@ -2996,7 +2995,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A10" s="5" t="s">
+      <c r="A10" t="s">
         <v>209</v>
       </c>
       <c r="B10" t="s">
@@ -3010,7 +3009,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" s="5" t="s">
+      <c r="A11" t="s">
         <v>211</v>
       </c>
       <c r="B11" t="s">
@@ -3024,7 +3023,7 @@
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A12" s="5" t="s">
+      <c r="A12" t="s">
         <v>213</v>
       </c>
       <c r="B12" t="s">
@@ -3038,12 +3037,12 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" s="5" t="s">
+      <c r="A13" t="s">
         <v>215</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14" s="5" t="s">
+      <c r="A14" t="s">
         <v>216</v>
       </c>
       <c r="B14" t="s">
@@ -3057,7 +3056,7 @@
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A15" s="5" t="s">
+      <c r="A15" t="s">
         <v>218</v>
       </c>
       <c r="B15" t="s">
@@ -3071,7 +3070,7 @@
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A16" s="5" t="s">
+      <c r="A16" t="s">
         <v>220</v>
       </c>
       <c r="B16" t="s">
@@ -3085,7 +3084,7 @@
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17" s="5" t="s">
+      <c r="A17" t="s">
         <v>199</v>
       </c>
       <c r="B17" t="s">
@@ -3099,12 +3098,12 @@
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18" s="5" t="s">
+      <c r="A18" t="s">
         <v>222</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A19" s="5" t="s">
+      <c r="A19" t="s">
         <v>223</v>
       </c>
       <c r="B19" t="s">
@@ -3118,7 +3117,7 @@
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A20" s="5" t="s">
+      <c r="A20" t="s">
         <v>225</v>
       </c>
       <c r="B20" t="s">
@@ -3132,7 +3131,7 @@
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A21" s="5" t="s">
+      <c r="A21" t="s">
         <v>227</v>
       </c>
       <c r="B21" t="s">
@@ -3146,7 +3145,7 @@
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A22" s="5" t="s">
+      <c r="A22" t="s">
         <v>229</v>
       </c>
       <c r="B22" t="s">
@@ -3160,7 +3159,7 @@
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A23" s="5" t="s">
+      <c r="A23" t="s">
         <v>231</v>
       </c>
       <c r="B23" t="s">
@@ -3174,7 +3173,7 @@
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A24" s="5" t="s">
+      <c r="A24" t="s">
         <v>233</v>
       </c>
       <c r="B24" t="s">
@@ -3188,12 +3187,12 @@
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A25" s="5" t="s">
+      <c r="A25" t="s">
         <v>235</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A26" s="5" t="s">
+      <c r="A26" t="s">
         <v>236</v>
       </c>
       <c r="B26" t="s">
@@ -3210,12 +3209,12 @@
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A27" s="5" t="s">
+      <c r="A27" t="s">
         <v>239</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A28" s="5" t="s">
+      <c r="A28" t="s">
         <v>240</v>
       </c>
       <c r="B28" t="s">
@@ -3232,7 +3231,7 @@
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A29" s="5" t="s">
+      <c r="A29" t="s">
         <v>244</v>
       </c>
       <c r="B29" t="s">
@@ -3249,7 +3248,7 @@
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A30" s="5" t="s">
+      <c r="A30" t="s">
         <v>246</v>
       </c>
       <c r="B30" t="s">
@@ -3266,12 +3265,12 @@
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A31" s="5" t="s">
+      <c r="A31" t="s">
         <v>247</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A32" s="5" t="s">
+      <c r="A32" t="s">
         <v>199</v>
       </c>
       <c r="B32" t="s">
@@ -3288,7 +3287,7 @@
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A33" s="5" t="s">
+      <c r="A33" t="s">
         <v>251</v>
       </c>
       <c r="B33" t="s">
@@ -3305,7 +3304,7 @@
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A34" s="5" t="s">
+      <c r="A34" t="s">
         <v>254</v>
       </c>
       <c r="B34" t="s">
@@ -3322,7 +3321,7 @@
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A35" s="5" t="s">
+      <c r="A35" t="s">
         <v>256</v>
       </c>
       <c r="B35" t="s">
@@ -3339,12 +3338,12 @@
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A36" s="5" t="s">
+      <c r="A36" t="s">
         <v>258</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A37" s="5" t="s">
+      <c r="A37" t="s">
         <v>125</v>
       </c>
       <c r="B37" t="s">
@@ -3358,7 +3357,7 @@
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A38" s="5" t="s">
+      <c r="A38" t="s">
         <v>260</v>
       </c>
       <c r="B38" t="s">
@@ -3375,7 +3374,7 @@
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A39" s="5" t="s">
+      <c r="A39" t="s">
         <v>263</v>
       </c>
       <c r="B39" t="s">
@@ -3392,7 +3391,7 @@
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A40" s="5" t="s">
+      <c r="A40" t="s">
         <v>265</v>
       </c>
       <c r="B40" t="s">
@@ -3409,7 +3408,7 @@
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A41" s="5" t="s">
+      <c r="A41" t="s">
         <v>268</v>
       </c>
       <c r="B41" t="s">
@@ -3426,7 +3425,7 @@
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A42" s="5" t="s">
+      <c r="A42" t="s">
         <v>271</v>
       </c>
       <c r="B42" t="s">
@@ -3443,7 +3442,7 @@
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A43" s="5" t="s">
+      <c r="A43" t="s">
         <v>273</v>
       </c>
       <c r="B43" t="s">
@@ -3611,7 +3610,7 @@
         <v>296</v>
       </c>
       <c r="C10">
-        <v>1.1000000000000001</v>
+        <v>1.05</v>
       </c>
       <c r="D10" t="s">
         <v>8</v>

</xml_diff>